<commit_message>
feat(engineering): close scoped power import calculation and release workflow
</commit_message>
<xml_diff>
--- a/dev/backend/internal/engineering/testdata/five-step/05-power.xlsx
+++ b/dev/backend/internal/engineering/testdata/five-step/05-power.xlsx
@@ -7,18 +7,43 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="power_profiles" sheetId="2" r:id="rId4"/>
-    <sheet name="rack_capacity" sheetId="3" r:id="rId6"/>
-    <sheet name="power_circuits" sheetId="4" r:id="rId7"/>
-    <sheet name="power_connections" sheetId="5" r:id="rId8"/>
-    <sheet name="power_rules" sheetId="6" r:id="rId9"/>
+    <sheet name="power_scope" sheetId="2" r:id="rId4"/>
+    <sheet name="power_profiles" sheetId="3" r:id="rId6"/>
+    <sheet name="rack_capacity" sheetId="4" r:id="rId7"/>
+    <sheet name="power_circuits" sheetId="5" r:id="rId8"/>
+    <sheet name="power_connections" sheetId="6" r:id="rId9"/>
+    <sheet name="power_rules" sheetId="7" r:id="rId10"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+  <si>
+    <t>场景</t>
+  </si>
+  <si>
+    <t>功率依据</t>
+  </si>
+  <si>
+    <t>需求规则引用</t>
+  </si>
+  <si>
+    <t>冗余要求</t>
+  </si>
+  <si>
+    <t>normal-single-feed</t>
+  </si>
+  <si>
+    <t>planned</t>
+  </si>
+  <si>
+    <t>fixture-power@1</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
   <si>
     <t>设备SN或型号引用</t>
   </si>
@@ -29,9 +54,6 @@
     <t>功率单位</t>
   </si>
   <si>
-    <t>功率依据</t>
-  </si>
-  <si>
     <t>来源</t>
   </si>
   <si>
@@ -44,9 +66,6 @@
     <t>W</t>
   </si>
   <si>
-    <t>planned</t>
-  </si>
-  <si>
     <t>SYNTHETIC_ONLY engineering input</t>
   </si>
   <si>
@@ -137,9 +156,6 @@
     <t>A</t>
   </si>
   <si>
-    <t>fixture-full-load-v1</t>
-  </si>
-  <si>
     <t>规则编码</t>
   </si>
   <si>
@@ -159,9 +175,6 @@
   </si>
   <si>
     <t>1</t>
-  </si>
-  <si>
-    <t>normal-single-feed</t>
   </si>
   <si>
     <t>SYNTHETIC_ONLY; not a redundant power design</t>
@@ -473,129 +486,97 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
+    <col max="4" min="1" style="1" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
     <col max="5" min="1" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="E2" s="1" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
-  <cols>
-    <col max="6" min="1" style="1" width="9.140625"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -611,62 +592,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -674,6 +655,77 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col max="6" min="1" style="1" width="9.140625"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
@@ -682,60 +734,60 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>39</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
   <cols>
@@ -744,42 +796,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>47</v>
+        <v>4</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>